<commit_message>
KneuHIRE sync 2026-05-21 21:29 UTC
</commit_message>
<xml_diff>
--- a/DATA.xlsx
+++ b/DATA.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -525,9 +525,57 @@
         <v>2026-05-21T21:27:03.945Z</v>
       </c>
     </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>JOB-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Regulatory Policy Specialist</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Policy Research / AI Governance</v>
+      </c>
+      <c r="D4" t="str">
+        <v>4+ years</v>
+      </c>
+      <c r="E4" t="str">
+        <v>₹20–35 LPA or equivalent</v>
+      </c>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Monitor global AI regulatory and standards developments
+Track updates related to the EU AI Act, NIST AI RMF, and ISO/IEC 42001
+Analyze sector-specific AI guidance, policies, and compliance expectations
+Translate regulatory developments into actionable business implications for clients
+Prepare policy briefings, risk summaries, and regulatory update reports
+Support internal advisory teams with governance and compliance insights
+Maintain regulatory intelligence repositories and tracking systems</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Strong understanding of AI governance and regulatory frameworks
+Deep familiarity with NIST AI RMF, ISO/IEC 42001, and EU AI Act requirements
+Ability to interpret legal, regulatory, and standards documentation
+Excellent research, analysis, and written communication skills
+Experience translating policy language into operational guidance
+Strong attention to detail and ability to track evolving regulations across jurisdictions</v>
+      </c>
+      <c r="H4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Background in technology policy, compliance, risk, or governance consulting
+Familiarity with emerging global AI regulations and standards bodies
+Experience working with enterprise compliance or legal teams
+Understanding of AI lifecycle management and responsible AI practices</v>
+      </c>
+      <c r="I4" t="str" xml:space="preserve">
+        <v xml:space="preserve">This role is ideal for someone who enjoys staying ahead of fast-moving regulatory developments and turning complex policy changes into practical guidance for organizations. The candidate should be highly analytical, research-driven, and capable of communicating nuanced regulatory insights clearly to both technical and non-technical stakeholders.
+CORE FRAMEWORKS &amp; STANDARDS
+NIST AI RMF · ISO/IEC 42001 · EU AI Act</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-05-21T21:29:12.081Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -556,7 +604,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2">
         <v>0</v>

</xml_diff>

<commit_message>
KneuHIRE sync 2026-05-21 21:32 UTC
</commit_message>
<xml_diff>
--- a/DATA.xlsx
+++ b/DATA.xlsx
@@ -582,10 +582,141 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData/>
+  <dimension ref="A1:U2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>role</v>
+      </c>
+      <c r="D1" t="str">
+        <v>dept</v>
+      </c>
+      <c r="E1" t="str">
+        <v>email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>intType</v>
+      </c>
+      <c r="G1" t="str">
+        <v>date</v>
+      </c>
+      <c r="H1" t="str">
+        <v>jobId</v>
+      </c>
+      <c r="I1" t="str">
+        <v>jobTitle</v>
+      </c>
+      <c r="J1" t="str">
+        <v>recommendation</v>
+      </c>
+      <c r="K1" t="str">
+        <v>avgScore</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ratedCount</v>
+      </c>
+      <c r="M1" t="str">
+        <v>overallNotes</v>
+      </c>
+      <c r="N1" t="str">
+        <v>recReason</v>
+      </c>
+      <c r="O1" t="str">
+        <v>submittedAt</v>
+      </c>
+      <c r="P1" t="str">
+        <v>score_tech</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>score_comm</v>
+      </c>
+      <c r="R1" t="str">
+        <v>score_prob</v>
+      </c>
+      <c r="S1" t="str">
+        <v>score_cult</v>
+      </c>
+      <c r="T1" t="str">
+        <v>score_lead</v>
+      </c>
+      <c r="U1" t="str">
+        <v>score_grow</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>CAND-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Piyal Gupta</v>
+      </c>
+      <c r="C2" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Corporate Functions</v>
+      </c>
+      <c r="E2" t="str">
+        <v>piyal@outlook.com</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Final Round</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="H2" t="str">
+        <v>—</v>
+      </c>
+      <c r="I2" t="str">
+        <v>CEO</v>
+      </c>
+      <c r="J2" t="str">
+        <v>hire</v>
+      </c>
+      <c r="K2" t="str">
+        <v>4.5</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-05-21T21:32:32.281Z</v>
+      </c>
+      <c r="P2">
+        <v>4</v>
+      </c>
+      <c r="Q2">
+        <v>4</v>
+      </c>
+      <c r="R2">
+        <v>4</v>
+      </c>
+      <c r="S2">
+        <v>5</v>
+      </c>
+      <c r="T2">
+        <v>5</v>
+      </c>
+      <c r="U2">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -607,7 +738,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>